<commit_message>
Update HOTAS Switch and Button - Quick Reference - ENHANCED - T16000.xlsx
Updated with latest testing results
</commit_message>
<xml_diff>
--- a/MapFiles/HOTAS Switch and Button - Quick Reference - ENHANCED - T16000.xlsx
+++ b/MapFiles/HOTAS Switch and Button - Quick Reference - ENHANCED - T16000.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Den\OneDrive\Personal\Thrustmaster\TARGET\Clicker\Development\ED_Enhanced_T16000\MapFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D5420C6-3A63-4664-A8E1-B2612A098456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1691218C-F631-4034-90B8-1A66D79003A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11265" yWindow="720" windowWidth="24870" windowHeight="20235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5595" yWindow="450" windowWidth="19725" windowHeight="20235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1269,7 +1269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1454,13 +1454,52 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1525,48 +1564,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1874,17 +1871,17 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="92" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="81"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="94"/>
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2"/>
@@ -1899,18 +1896,18 @@
       <c r="O3"/>
     </row>
     <row r="4" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="76" t="s">
+      <c r="B4" s="89" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="77"/>
-      <c r="D4" s="77"/>
-      <c r="E4" s="78"/>
-      <c r="G4" s="76" t="s">
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="91"/>
+      <c r="G4" s="89" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="77"/>
-      <c r="I4" s="77"/>
-      <c r="J4" s="78"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="91"/>
       <c r="K4"/>
       <c r="L4"/>
       <c r="M4"/>
@@ -1961,7 +1958,7 @@
       <c r="C7" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="98" t="s">
+      <c r="D7" s="76" t="s">
         <v>54</v>
       </c>
       <c r="E7" s="25" t="s">
@@ -1973,7 +1970,7 @@
       <c r="H7" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="I7" s="98" t="s">
+      <c r="I7" s="76" t="s">
         <v>57</v>
       </c>
       <c r="J7" s="25" t="s">
@@ -1991,7 +1988,7 @@
       <c r="C8" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="86" t="s">
+      <c r="D8" s="64" t="s">
         <v>55</v>
       </c>
       <c r="E8" s="3" t="s">
@@ -2003,7 +2000,7 @@
       <c r="H8" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="I8" s="86" t="s">
+      <c r="I8" s="64" t="s">
         <v>56</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -2021,7 +2018,7 @@
       <c r="C9" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="86" t="s">
+      <c r="D9" s="64" t="s">
         <v>56</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -2033,7 +2030,7 @@
       <c r="H9" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="I9" s="86" t="s">
+      <c r="I9" s="64" t="s">
         <v>58</v>
       </c>
       <c r="J9" s="3" t="s">
@@ -2061,7 +2058,7 @@
       <c r="H10" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="I10" s="86" t="s">
+      <c r="I10" s="64" t="s">
         <v>59</v>
       </c>
       <c r="J10" s="3" t="s">
@@ -2079,7 +2076,7 @@
       <c r="H11" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="I11" s="99" t="s">
+      <c r="I11" s="77" t="s">
         <v>71</v>
       </c>
       <c r="J11" s="5" t="s">
@@ -2119,7 +2116,7 @@
     </row>
     <row r="14" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="65" t="s">
+      <c r="B15" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="11" t="s">
@@ -2131,34 +2128,34 @@
       <c r="E15" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="G15" s="69" t="s">
+      <c r="G15" s="82" t="s">
         <v>26</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="I15" s="89" t="s">
+      <c r="I15" s="67" t="s">
         <v>137</v>
       </c>
       <c r="J15" s="13"/>
       <c r="L15" s="9"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="66"/>
+      <c r="B16" s="79"/>
       <c r="C16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="86" t="s">
+      <c r="D16" s="64" t="s">
         <v>106</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G16" s="70"/>
+      <c r="G16" s="83"/>
       <c r="H16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I16" s="90" t="s">
+      <c r="I16" s="68" t="s">
         <v>119</v>
       </c>
       <c r="J16" s="16" t="s">
@@ -2167,17 +2164,17 @@
       <c r="L16" s="9"/>
     </row>
     <row r="17" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="67"/>
+      <c r="B17" s="80"/>
       <c r="C17" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="87" t="s">
+      <c r="D17" s="65" t="s">
         <v>87</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="G17" s="71"/>
+      <c r="G17" s="84"/>
       <c r="H17" s="6" t="s">
         <v>64</v>
       </c>
@@ -2200,7 +2197,7 @@
       </c>
     </row>
     <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="65" t="s">
+      <c r="B19" s="78" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="11" t="s">
@@ -2227,17 +2224,17 @@
       <c r="L19" s="9"/>
     </row>
     <row r="20" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="66"/>
+      <c r="B20" s="79"/>
       <c r="C20" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="64" t="s">
         <v>108</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="72" t="s">
+      <c r="G20" s="85" t="s">
         <v>29</v>
       </c>
       <c r="H20" s="29" t="s">
@@ -2248,7 +2245,7 @@
       <c r="L20" s="9"/>
     </row>
     <row r="21" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="67"/>
+      <c r="B21" s="80"/>
       <c r="C21" s="4" t="s">
         <v>64</v>
       </c>
@@ -2258,11 +2255,11 @@
       <c r="E21" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="73"/>
+      <c r="G21" s="86"/>
       <c r="H21" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="I21" s="86" t="s">
+      <c r="I21" s="64" t="s">
         <v>141</v>
       </c>
       <c r="J21" s="16" t="s">
@@ -2271,7 +2268,7 @@
     </row>
     <row r="22" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="9"/>
-      <c r="G22" s="74"/>
+      <c r="G22" s="87"/>
       <c r="H22" s="38" t="s">
         <v>64</v>
       </c>
@@ -2284,19 +2281,19 @@
       <c r="L22" s="9"/>
     </row>
     <row r="23" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="65" t="s">
+      <c r="B23" s="78" t="s">
         <v>12</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="88" t="s">
+      <c r="D23" s="66" t="s">
         <v>111</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="G23" s="73" t="s">
+      <c r="G23" s="86" t="s">
         <v>30</v>
       </c>
       <c r="H23" s="39" t="s">
@@ -2309,37 +2306,37 @@
       <c r="L23" s="9"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="66"/>
+      <c r="B24" s="79"/>
       <c r="C24" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="86" t="s">
+      <c r="D24" s="64" t="s">
         <v>109</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="G24" s="73"/>
+      <c r="G24" s="86"/>
       <c r="H24" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I24" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="J24" s="64"/>
+      <c r="J24" s="63"/>
     </row>
     <row r="25" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="67"/>
+      <c r="B25" s="80"/>
       <c r="C25" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="77" t="s">
         <v>151</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="G25" s="75"/>
+      <c r="G25" s="88"/>
       <c r="H25" s="17" t="s">
         <v>64</v>
       </c>
@@ -2356,19 +2353,19 @@
       <c r="I26" s="30"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B27" s="65" t="s">
+      <c r="B27" s="78" t="s">
         <v>13</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="67" t="s">
         <v>91</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="G27" s="65" t="s">
+      <c r="G27" s="78" t="s">
         <v>31</v>
       </c>
       <c r="H27" s="11" t="s">
@@ -2379,21 +2376,21 @@
       <c r="L27" s="9"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="66"/>
+      <c r="B28" s="79"/>
       <c r="C28" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="62" t="s">
+      <c r="D28" s="72" t="s">
         <v>92</v>
       </c>
       <c r="E28" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="G28" s="66"/>
+      <c r="G28" s="79"/>
       <c r="H28" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I28" s="90" t="s">
+      <c r="I28" s="68" t="s">
         <v>120</v>
       </c>
       <c r="J28" s="3" t="s">
@@ -2401,17 +2398,17 @@
       </c>
     </row>
     <row r="29" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="67"/>
+      <c r="B29" s="80"/>
       <c r="C29" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="77" t="s">
         <v>113</v>
       </c>
       <c r="E29" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="G29" s="67"/>
+      <c r="G29" s="80"/>
       <c r="H29" s="4" t="s">
         <v>64</v>
       </c>
@@ -2427,7 +2424,7 @@
       <c r="L30" s="9"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="65" t="s">
+      <c r="B31" s="78" t="s">
         <v>0</v>
       </c>
       <c r="C31" s="11" t="s">
@@ -2437,13 +2434,13 @@
         <v>105</v>
       </c>
       <c r="E31" s="13"/>
-      <c r="G31" s="69" t="s">
+      <c r="G31" s="82" t="s">
         <v>32</v>
       </c>
       <c r="H31" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="I31" s="11" t="s">
+      <c r="I31" s="67" t="s">
         <v>121</v>
       </c>
       <c r="J31" s="13" t="s">
@@ -2452,19 +2449,19 @@
       <c r="P31" s="30"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="66"/>
+      <c r="B32" s="79"/>
       <c r="C32" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D32" s="86" t="s">
+      <c r="D32" s="64" t="s">
         <v>93</v>
       </c>
       <c r="E32" s="20"/>
-      <c r="G32" s="70"/>
+      <c r="G32" s="83"/>
       <c r="H32" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I32" s="86" t="s">
+      <c r="I32" s="64" t="s">
         <v>130</v>
       </c>
       <c r="J32" s="3" t="s">
@@ -2474,7 +2471,7 @@
       <c r="P32" s="30"/>
     </row>
     <row r="33" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="68"/>
+      <c r="B33" s="81"/>
       <c r="C33" s="34" t="s">
         <v>64</v>
       </c>
@@ -2482,7 +2479,7 @@
         <v>98</v>
       </c>
       <c r="E33" s="35"/>
-      <c r="G33" s="71"/>
+      <c r="G33" s="84"/>
       <c r="H33" s="6" t="s">
         <v>64</v>
       </c>
@@ -2494,7 +2491,7 @@
       <c r="P33" s="30"/>
     </row>
     <row r="34" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="66" t="s">
+      <c r="B34" s="79" t="s">
         <v>1</v>
       </c>
       <c r="C34" s="19" t="s">
@@ -2504,7 +2501,7 @@
         <v>97</v>
       </c>
       <c r="E34" s="20"/>
-      <c r="G34" s="82" t="s">
+      <c r="G34" s="95" t="s">
         <v>33</v>
       </c>
       <c r="H34" s="29" t="s">
@@ -2519,7 +2516,7 @@
       <c r="P34" s="30"/>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B35" s="66"/>
+      <c r="B35" s="79"/>
       <c r="C35" s="2" t="s">
         <v>62</v>
       </c>
@@ -2529,11 +2526,11 @@
       <c r="E35" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="G35" s="70"/>
+      <c r="G35" s="83"/>
       <c r="H35" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I35" s="86" t="s">
+      <c r="I35" s="64" t="s">
         <v>131</v>
       </c>
       <c r="J35" s="3" t="s">
@@ -2543,7 +2540,7 @@
       <c r="P35" s="30"/>
     </row>
     <row r="36" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="68"/>
+      <c r="B36" s="81"/>
       <c r="C36" s="6" t="s">
         <v>64</v>
       </c>
@@ -2551,7 +2548,7 @@
         <v>96</v>
       </c>
       <c r="E36" s="7"/>
-      <c r="G36" s="71"/>
+      <c r="G36" s="84"/>
       <c r="H36" s="6" t="s">
         <v>64</v>
       </c>
@@ -2562,19 +2559,19 @@
       <c r="Q36" s="8"/>
     </row>
     <row r="37" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="83" t="s">
+      <c r="B37" s="96" t="s">
         <v>2</v>
       </c>
       <c r="C37" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="D37" s="93" t="s">
+      <c r="D37" s="71" t="s">
         <v>115</v>
       </c>
       <c r="E37" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="G37" s="82" t="s">
+      <c r="G37" s="95" t="s">
         <v>34</v>
       </c>
       <c r="H37" s="29" t="s">
@@ -2588,19 +2585,19 @@
       <c r="Q37" s="8"/>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B38" s="66"/>
+      <c r="B38" s="79"/>
       <c r="C38" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D38" s="86" t="s">
+      <c r="D38" s="64" t="s">
         <v>94</v>
       </c>
       <c r="E38" s="3"/>
-      <c r="G38" s="70"/>
+      <c r="G38" s="83"/>
       <c r="H38" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I38" s="86" t="s">
+      <c r="I38" s="64" t="s">
         <v>132</v>
       </c>
       <c r="J38" s="3"/>
@@ -2609,17 +2606,17 @@
       <c r="Q38" s="8"/>
     </row>
     <row r="39" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="68"/>
+      <c r="B39" s="81"/>
       <c r="C39" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="91" t="s">
+      <c r="D39" s="69" t="s">
         <v>175</v>
       </c>
       <c r="E39" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="G39" s="71"/>
+      <c r="G39" s="84"/>
       <c r="H39" s="6" t="s">
         <v>64</v>
       </c>
@@ -2630,19 +2627,19 @@
       <c r="Q39" s="8"/>
     </row>
     <row r="40" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="83" t="s">
+      <c r="B40" s="96" t="s">
         <v>3</v>
       </c>
       <c r="C40" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="D40" s="19" t="s">
+      <c r="D40" s="71" t="s">
         <v>161</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="G40" s="84" t="s">
+      <c r="G40" s="97" t="s">
         <v>35</v>
       </c>
       <c r="H40" s="19" t="s">
@@ -2655,19 +2652,19 @@
       <c r="P40" s="30"/>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B41" s="66"/>
+      <c r="B41" s="79"/>
       <c r="C41" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="D41" s="64" t="s">
         <v>116</v>
       </c>
       <c r="E41" s="3"/>
-      <c r="G41" s="70"/>
+      <c r="G41" s="83"/>
       <c r="H41" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I41" s="86" t="s">
+      <c r="I41" s="64" t="s">
         <v>133</v>
       </c>
       <c r="J41" s="3" t="s">
@@ -2677,17 +2674,17 @@
       <c r="P41" s="30"/>
     </row>
     <row r="42" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="67"/>
+      <c r="B42" s="80"/>
       <c r="C42" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="77" t="s">
         <v>160</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="G42" s="85"/>
+      <c r="G42" s="98"/>
       <c r="H42" s="4" t="s">
         <v>64</v>
       </c>
@@ -2702,7 +2699,7 @@
       <c r="P43" s="30"/>
     </row>
     <row r="44" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B44" s="69" t="s">
+      <c r="B44" s="82" t="s">
         <v>14</v>
       </c>
       <c r="C44" s="11" t="s">
@@ -2710,13 +2707,13 @@
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="13"/>
-      <c r="G44" s="69" t="s">
+      <c r="G44" s="82" t="s">
         <v>36</v>
       </c>
       <c r="H44" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="I44" s="89" t="s">
+      <c r="I44" s="67" t="s">
         <v>143</v>
       </c>
       <c r="J44" s="13" t="s">
@@ -2726,19 +2723,19 @@
       <c r="P44" s="30"/>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B45" s="70"/>
+      <c r="B45" s="83"/>
       <c r="C45" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D45" s="86" t="s">
+      <c r="D45" s="64" t="s">
         <v>99</v>
       </c>
       <c r="E45" s="3"/>
-      <c r="G45" s="70"/>
+      <c r="G45" s="83"/>
       <c r="H45" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I45" s="86" t="s">
+      <c r="I45" s="64" t="s">
         <v>124</v>
       </c>
       <c r="J45" s="3" t="s">
@@ -2747,17 +2744,17 @@
       <c r="L45" s="9"/>
     </row>
     <row r="46" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="71"/>
+      <c r="B46" s="84"/>
       <c r="C46" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="7"/>
-      <c r="G46" s="71"/>
+      <c r="G46" s="84"/>
       <c r="H46" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I46" s="91" t="s">
+      <c r="I46" s="69" t="s">
         <v>144</v>
       </c>
       <c r="J46" s="7" t="s">
@@ -2765,7 +2762,7 @@
       </c>
     </row>
     <row r="47" spans="2:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="82" t="s">
+      <c r="B47" s="95" t="s">
         <v>15</v>
       </c>
       <c r="C47" s="29" t="s">
@@ -2773,13 +2770,13 @@
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="36"/>
-      <c r="G47" s="82" t="s">
+      <c r="G47" s="95" t="s">
         <v>37</v>
       </c>
       <c r="H47" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="I47" s="92" t="s">
+      <c r="I47" s="70" t="s">
         <v>145</v>
       </c>
       <c r="J47" s="36" t="s">
@@ -2788,21 +2785,21 @@
       <c r="L47" s="9"/>
     </row>
     <row r="48" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B48" s="70"/>
+      <c r="B48" s="83"/>
       <c r="C48" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="D48" s="64" t="s">
         <v>197</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="G48" s="70"/>
+      <c r="G48" s="83"/>
       <c r="H48" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I48" s="86" t="s">
+      <c r="I48" s="64" t="s">
         <v>125</v>
       </c>
       <c r="J48" s="3" t="s">
@@ -2811,13 +2808,13 @@
       <c r="L48" s="9"/>
     </row>
     <row r="49" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="71"/>
+      <c r="B49" s="84"/>
       <c r="C49" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="7"/>
-      <c r="G49" s="71"/>
+      <c r="G49" s="84"/>
       <c r="H49" s="6" t="s">
         <v>64</v>
       </c>
@@ -2825,7 +2822,7 @@
       <c r="J49" s="7"/>
     </row>
     <row r="50" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="82" t="s">
+      <c r="B50" s="95" t="s">
         <v>16</v>
       </c>
       <c r="C50" s="29" t="s">
@@ -2833,7 +2830,7 @@
       </c>
       <c r="D50" s="29"/>
       <c r="E50" s="36"/>
-      <c r="G50" s="82" t="s">
+      <c r="G50" s="95" t="s">
         <v>38</v>
       </c>
       <c r="H50" s="29" t="s">
@@ -2845,21 +2842,21 @@
       <c r="J50" s="36"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="70"/>
+      <c r="B51" s="83"/>
       <c r="C51" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D51" s="86" t="s">
+      <c r="D51" s="64" t="s">
         <v>100</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="G51" s="70"/>
+      <c r="G51" s="83"/>
       <c r="H51" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I51" s="86" t="s">
+      <c r="I51" s="64" t="s">
         <v>126</v>
       </c>
       <c r="J51" s="3" t="s">
@@ -2867,13 +2864,13 @@
       </c>
     </row>
     <row r="52" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="71"/>
+      <c r="B52" s="84"/>
       <c r="C52" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="7"/>
-      <c r="G52" s="71"/>
+      <c r="G52" s="84"/>
       <c r="H52" s="6" t="s">
         <v>64</v>
       </c>
@@ -2881,7 +2878,7 @@
       <c r="J52" s="7"/>
     </row>
     <row r="53" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="82" t="s">
+      <c r="B53" s="95" t="s">
         <v>17</v>
       </c>
       <c r="C53" s="29" t="s">
@@ -2889,7 +2886,7 @@
       </c>
       <c r="D53" s="29"/>
       <c r="E53" s="36"/>
-      <c r="G53" s="84" t="s">
+      <c r="G53" s="97" t="s">
         <v>39</v>
       </c>
       <c r="H53" s="19" t="s">
@@ -2901,21 +2898,21 @@
       <c r="J53" s="20"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B54" s="70"/>
+      <c r="B54" s="83"/>
       <c r="C54" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D54" s="86" t="s">
+      <c r="D54" s="64" t="s">
         <v>156</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="G54" s="70"/>
+      <c r="G54" s="83"/>
       <c r="H54" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I54" s="86" t="s">
+      <c r="I54" s="64" t="s">
         <v>127</v>
       </c>
       <c r="J54" s="3" t="s">
@@ -2923,13 +2920,13 @@
       </c>
     </row>
     <row r="55" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="71"/>
+      <c r="B55" s="84"/>
       <c r="C55" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="7"/>
-      <c r="G55" s="85"/>
+      <c r="G55" s="98"/>
       <c r="H55" s="4" t="s">
         <v>64</v>
       </c>
@@ -2937,7 +2934,7 @@
       <c r="J55" s="5"/>
     </row>
     <row r="56" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="82" t="s">
+      <c r="B56" s="95" t="s">
         <v>18</v>
       </c>
       <c r="C56" s="29" t="s">
@@ -2947,7 +2944,7 @@
       <c r="E56" s="36"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="70"/>
+      <c r="B57" s="83"/>
       <c r="C57" s="2" t="s">
         <v>62</v>
       </c>
@@ -2957,7 +2954,7 @@
       <c r="E57" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="G57" s="69" t="s">
+      <c r="G57" s="82" t="s">
         <v>40</v>
       </c>
       <c r="H57" s="11" t="s">
@@ -2971,13 +2968,13 @@
       </c>
     </row>
     <row r="58" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="71"/>
+      <c r="B58" s="84"/>
       <c r="C58" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="7"/>
-      <c r="G58" s="70"/>
+      <c r="G58" s="83"/>
       <c r="H58" s="2" t="s">
         <v>62</v>
       </c>
@@ -2989,7 +2986,7 @@
       </c>
     </row>
     <row r="59" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="84" t="s">
+      <c r="B59" s="97" t="s">
         <v>19</v>
       </c>
       <c r="C59" s="19" t="s">
@@ -2997,7 +2994,7 @@
       </c>
       <c r="D59" s="19"/>
       <c r="E59" s="20"/>
-      <c r="G59" s="71"/>
+      <c r="G59" s="84"/>
       <c r="H59" s="6" t="s">
         <v>64</v>
       </c>
@@ -3009,15 +3006,15 @@
       </c>
     </row>
     <row r="60" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="70"/>
+      <c r="B60" s="83"/>
       <c r="C60" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D60" s="94" t="s">
+      <c r="D60" s="72" t="s">
         <v>101</v>
       </c>
       <c r="E60" s="3"/>
-      <c r="G60" s="82" t="s">
+      <c r="G60" s="95" t="s">
         <v>41</v>
       </c>
       <c r="H60" s="29" t="s">
@@ -3027,17 +3024,17 @@
       <c r="J60" s="36"/>
     </row>
     <row r="61" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="85"/>
+      <c r="B61" s="98"/>
       <c r="C61" s="4" t="s">
         <v>64</v>
       </c>
       <c r="D61" s="4"/>
       <c r="E61" s="5"/>
-      <c r="G61" s="70"/>
+      <c r="G61" s="83"/>
       <c r="H61" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I61" s="2" t="s">
+      <c r="I61" s="64" t="s">
         <v>146</v>
       </c>
       <c r="J61" s="3" t="s">
@@ -3045,7 +3042,7 @@
       </c>
     </row>
     <row r="62" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G62" s="71"/>
+      <c r="G62" s="84"/>
       <c r="H62" s="6" t="s">
         <v>64</v>
       </c>
@@ -3053,15 +3050,15 @@
       <c r="J62" s="7"/>
     </row>
     <row r="63" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="69" t="s">
+      <c r="B63" s="82" t="s">
         <v>20</v>
       </c>
       <c r="C63" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D63" s="63"/>
+      <c r="D63" s="62"/>
       <c r="E63" s="13"/>
-      <c r="G63" s="82" t="s">
+      <c r="G63" s="95" t="s">
         <v>42</v>
       </c>
       <c r="H63" s="29" t="s">
@@ -3071,19 +3068,19 @@
       <c r="J63" s="36"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="70"/>
+      <c r="B64" s="83"/>
       <c r="C64" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D64" s="86" t="s">
+      <c r="D64" s="64" t="s">
         <v>182</v>
       </c>
       <c r="E64" s="3"/>
-      <c r="G64" s="70"/>
+      <c r="G64" s="83"/>
       <c r="H64" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I64" s="2" t="s">
+      <c r="I64" s="64" t="s">
         <v>147</v>
       </c>
       <c r="J64" s="3" t="s">
@@ -3091,13 +3088,13 @@
       </c>
     </row>
     <row r="65" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="71"/>
+      <c r="B65" s="84"/>
       <c r="C65" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="7"/>
-      <c r="G65" s="71"/>
+      <c r="G65" s="84"/>
       <c r="H65" s="6" t="s">
         <v>64</v>
       </c>
@@ -3105,7 +3102,7 @@
       <c r="J65" s="7"/>
     </row>
     <row r="66" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="82" t="s">
+      <c r="B66" s="95" t="s">
         <v>21</v>
       </c>
       <c r="C66" s="29" t="s">
@@ -3113,7 +3110,7 @@
       </c>
       <c r="D66" s="29"/>
       <c r="E66" s="36"/>
-      <c r="G66" s="84" t="s">
+      <c r="G66" s="97" t="s">
         <v>43</v>
       </c>
       <c r="H66" s="19" t="s">
@@ -3123,13 +3120,13 @@
       <c r="J66" s="20"/>
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B67" s="70"/>
+      <c r="B67" s="83"/>
       <c r="C67" s="2" t="s">
         <v>62</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="3"/>
-      <c r="G67" s="70"/>
+      <c r="G67" s="83"/>
       <c r="H67" s="2" t="s">
         <v>62</v>
       </c>
@@ -3141,13 +3138,13 @@
       </c>
     </row>
     <row r="68" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="71"/>
+      <c r="B68" s="84"/>
       <c r="C68" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="7"/>
-      <c r="G68" s="85"/>
+      <c r="G68" s="98"/>
       <c r="H68" s="4" t="s">
         <v>64</v>
       </c>
@@ -3155,7 +3152,7 @@
       <c r="J68" s="5"/>
     </row>
     <row r="69" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="82" t="s">
+      <c r="B69" s="95" t="s">
         <v>22</v>
       </c>
       <c r="C69" s="29" t="s">
@@ -3165,25 +3162,25 @@
       <c r="E69" s="36"/>
     </row>
     <row r="70" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="70"/>
+      <c r="B70" s="83"/>
       <c r="C70" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D70" s="86" t="s">
+      <c r="D70" s="64" t="s">
         <v>183</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="G70" s="76" t="s">
+      <c r="G70" s="89" t="s">
         <v>77</v>
       </c>
-      <c r="H70" s="77"/>
-      <c r="I70" s="77"/>
-      <c r="J70" s="78"/>
+      <c r="H70" s="90"/>
+      <c r="I70" s="90"/>
+      <c r="J70" s="91"/>
     </row>
     <row r="71" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="71"/>
+      <c r="B71" s="84"/>
       <c r="C71" s="6" t="s">
         <v>64</v>
       </c>
@@ -3191,7 +3188,7 @@
       <c r="E71" s="7"/>
     </row>
     <row r="72" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="82" t="s">
+      <c r="B72" s="95" t="s">
         <v>23</v>
       </c>
       <c r="C72" s="29" t="s">
@@ -3215,7 +3212,7 @@
       </c>
     </row>
     <row r="73" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="70"/>
+      <c r="B73" s="83"/>
       <c r="C73" s="2" t="s">
         <v>62</v>
       </c>
@@ -3229,7 +3226,7 @@
       <c r="H73" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="I73" s="86" t="s">
+      <c r="I73" s="64" t="s">
         <v>56</v>
       </c>
       <c r="J73" s="25" t="s">
@@ -3237,7 +3234,7 @@
       </c>
     </row>
     <row r="74" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="71"/>
+      <c r="B74" s="84"/>
       <c r="C74" s="6" t="s">
         <v>64</v>
       </c>
@@ -3257,7 +3254,7 @@
       <c r="J74" s="3"/>
     </row>
     <row r="75" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="82" t="s">
+      <c r="B75" s="95" t="s">
         <v>24</v>
       </c>
       <c r="C75" s="29" t="s">
@@ -3277,7 +3274,7 @@
       <c r="J75" s="5"/>
     </row>
     <row r="76" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="70"/>
+      <c r="B76" s="83"/>
       <c r="C76" s="2" t="s">
         <v>62</v>
       </c>
@@ -3293,7 +3290,7 @@
       <c r="J76" s="58"/>
     </row>
     <row r="77" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="71"/>
+      <c r="B77" s="84"/>
       <c r="C77" s="6" t="s">
         <v>64</v>
       </c>
@@ -3313,13 +3310,13 @@
       </c>
     </row>
     <row r="78" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="84" t="s">
+      <c r="B78" s="97" t="s">
         <v>25</v>
       </c>
       <c r="C78" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D78" s="95" t="s">
+      <c r="D78" s="73" t="s">
         <v>139</v>
       </c>
       <c r="E78" s="20" t="s">
@@ -3337,11 +3334,11 @@
       <c r="J78" s="3"/>
     </row>
     <row r="79" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B79" s="70"/>
+      <c r="B79" s="83"/>
       <c r="C79" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D79" s="96" t="s">
+      <c r="D79" s="74" t="s">
         <v>140</v>
       </c>
       <c r="E79" s="3" t="s">
@@ -3359,11 +3356,11 @@
       <c r="J79" s="5"/>
     </row>
     <row r="80" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="85"/>
+      <c r="B80" s="98"/>
       <c r="C80" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D80" s="97" t="s">
+      <c r="D80" s="75" t="s">
         <v>138</v>
       </c>
       <c r="E80" s="5" t="s">

</xml_diff>